<commit_message>
feat(F-NAR-019): ATOM-AUT.AFF.001-05 L'escargot du jardin
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.AFF.001-05.xlsx
+++ b/stories/arbres/ATOM-AUT.AFF.001-05.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>maison puis jardin après la pluie</t>
+          <t>maison puis le coin du seau, jardin après la pluie</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Raphaël veut l'escargot du jardin après la pluie. Le zip résiste. Il pousse, glisse le livre, trouve la coquille brillante.</t>
+          <t>Raphaël veut voir l'escargot du coin du seau avant que sa trace sèche. Il fonce, le zip se coince sur un grain de feuille. Il refuse de tirer, glisse la loupe dans le sac, retrouve le même grain sous la feuille du seau.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Une feuille mouillée colle au seau. Le jardin sent la terre après la pluie. Une goutte tombe encore d'une branche. Elle fait un petit cercle dans une flaque. Papa ouvre le tiroir de laine. Ça fait un petit bruit. Les vitres sont un peu grises. Une tasse fume près de la fenêtre. Raphaël, tu entends la goutte ? Oui. Je veux l'escargot. Il est dans le jardin, tout lent. On y va, avec le sac. En ce moment, Raphaël s'accroupit. Le sac vert est par terre. Le tissu est un peu rêche. Il est vert, papa. Oui, c'est le tien. Prends de l'eau, même s'il a plu. Raphaël prend la gourde. Elle est froide comme la pluie. Il la met dans le sac. Le bonnet aussi, le vent est humide. Raphaël prend le bonnet. Il est tout doux. Il sent la laine du tiroir. Il est chaud. Il le met dans le sac. Et le livre, si on s'assoit. Le livre est près de la tasse. La couverture est lisse. Une goutte glisse encore sur la vitre. Raphaël tire le zip. Le zip reste un peu. Ça ne veut pas, papa. Doucement, tu aides le zip ?</t>
+          <t>La vapeur de la tasse dessine un rond. Sur la vitre grise, le rond tremble. À travers, le seau jaune apparaît. Une feuille collée tapote au bord. Un grain de feuille brille dessus. Raphaël colle son nez à la vitre. Le jardin sent la terre mouillée. La dalle du seau luit, pâle. Papa ouvre le tiroir de laine. Ça fait un petit bruit sourd. La maison sent la laine et le thé. Une botte penche près de la porte. Raphaël, tu vois le grain dehors ? Oui, papa. Je veux l'escargot maintenant. Sa trace d'argent va sécher. On y va, avec le sac. En ce moment, Raphaël saisit le sac. Le sac vert est par terre. Une loupe ronde attend dans la poche. Il est vert, papa. Oui, c'est le tien. Prends la loupe, pour ses cornes. Raphaël prend la loupe ronde. Le verre est froid sous le doigt. Le bord fait un petit clic. Vite, il va partir. Raphaël tape du pied, impatient. Il pousse la loupe dans le sac. Il tire le zip d'un coup. Le zip se coince, dur. Ça ne veut pas, papa. La loupe bascule et glisse. Raphaël la rattrape contre sa poitrine. Son sourire disparaît. L'envie et l'inquiétude se bousculent. Le cœur de Raphaël bat plus fort. Papa s'accroupit à sa hauteur. Tu aides le zip ?</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Une feuille mouillée colle au seau. Le jardin sent la terre après la pluie. Une goutte tombe encore d'une branche. Elle fait un petit cercle dans une flaque. Papa ouvre le tiroir de laine. Ça fait un petit bruit. Les vitres sont un peu grises. Une tasse fume près de la fenêtre. Raphaël, tu entends la goutte ? Oui. Je veux l'escargot. Il est dans le jardin, tout lent. On y va, avec le sac. En ce moment, Raphaël s'accroupit. Le sac vert est par terre. Le tissu est un peu rêche. Il est vert, papa. Oui, c'est le tien. Prends de l'eau, même s'il a plu. Raphaël prend la gourde. Elle est froide comme la pluie. Il la met dans le sac. Le bonnet aussi, le vent est humide. Raphaël prend le bonnet. Il est tout doux. Il sent la laine du tiroir. Il est chaud. Il le met dans le sac. Et le livre, si on s'assoit. Le livre est près de la tasse. La couverture est lisse. Une goutte glisse encore sur la vitre. Raphaël tire le zip. Le zip reste un peu. Ça ne veut pas, papa. Doucement, tu aides le zip ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La vapeur de la tasse dessine un rond. Sur la vitre grise, le rond tremble. À travers, le seau jaune apparaît. Une feuille collée tapote au bord. Un &lt;emphasis level="moderate"&gt;grain de feuille&lt;/emphasis&gt; brille dessus. Raphaël colle son nez à la vitre. Le jardin sent la terre mouillée. La dalle du seau luit, pâle. Papa ouvre le tiroir de laine. Ça fait un petit bruit sourd. La maison sent la laine et le thé. Une botte penche près de la porte. Raphaël, tu vois le grain dehors ? Oui, papa. Je veux l'escargot maintenant. Sa trace d'argent va sécher. On y va, avec le sac. En ce moment, Raphaël saisit le sac. Le sac vert est par terre. Une loupe ronde attend dans la poche. Il est vert, papa. Oui, c'est le tien. Prends la loupe, pour ses cornes. Raphaël prend la loupe ronde. Le verre est froid sous le doigt. Le bord fait un petit clic. Vite, il va partir. Raphaël tape du pied, impatient. Il pousse la loupe dans le sac. Il tire le zip d'un coup. Le zip se coince, dur. Ça ne veut pas, papa. La loupe bascule et glisse. Raphaël la rattrape contre sa poitrine. Son sourire disparaît. L'envie et l'inquiétude se bousculent. Le cœur de Raphaël bat plus fort. Papa s'accroupit à sa hauteur. Tu aides le zip ?&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;C'est le matin. Xavier est dans l'entrée. Le &lt;emphasis&gt;sac&lt;/emphasis&gt; est par terre. Le sac est vert. Papa est là. Papa est l'adulte. Papa dit : la gourde, le bonnet, le livre. Xavier écoute. Il prend la gourde. Il la met dans le sac. Il prend le bonnet. Il le met dans le sac. Il prend le livre. Il le met dans le sac. Xavier ferme le sac. Ça fait zzz. Xavier a mis ce que l'adulte a dit. Papa dit : merci Xavier. Le sac est prêt.&lt;/slow&gt; [pause]</t>
+          <t>La vapeur de la tasse dessine un rond. Sur la vitre grise, le rond tremble. À travers, le seau jaune apparaît. Une feuille collée tapote au bord. Un &lt;emphasis&gt;grain de feuille&lt;/emphasis&gt; brille dessus. Raphaël colle son nez à la vitre. Le jardin sent la terre mouillée. La dalle du seau luit, pâle. Papa ouvre le tiroir de laine. Ça fait un petit bruit sourd. La maison sent la laine et le thé. Une botte penche près de la porte. Raphaël, tu vois le grain dehors ? Oui, papa. Je veux l'escargot maintenant. Sa trace d'argent va sécher. On y va, avec le sac. En ce moment, Raphaël saisit le sac. Le sac vert est par terre. Une loupe ronde attend dans la poche. Il est vert, papa. Oui, c'est le tien. Prends la loupe, pour ses cornes. Raphaël prend la loupe ronde. Le verre est froid sous le doigt. Le bord fait un petit clic. Vite, il va partir. Raphaël tape du pied, impatient. Il pousse la loupe dans le sac. Il tire le zip d'un coup. Le zip se coince, dur. Ça ne veut pas, papa. La loupe bascule et glisse. Raphaël la rattrape contre sa poitrine. Son sourire disparaît. L'envie et l'inquiétude se bousculent. Le cœur de Raphaël bat plus fort. Papa s'accroupit à sa hauteur. Tu aides le zip ? [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>sac</t>
+          <t>grain de feuille</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>380</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1319,52 +1319,59 @@
         <v>50</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller; emotion=impatience_curieuse; intensite=2; destinataire=enfant; sous_texte=le_grain_brille_sur_la_feuille_du_seau; tempo=naturel; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Une feuille mouillée colle au seau.
-narrateur|Le jardin sent la terre après la pluie.
-narrateur|Une goutte tombe encore d'une branche.
-narrateur|Elle fait un petit cercle dans une flaque.
+          <t>narrateur|La vapeur de la tasse dessine un rond.
+narrateur|Sur la vitre grise, le rond tremble.
+narrateur|À travers, le seau jaune apparaît.
+narrateur|Une feuille collée tapote au bord.
+narrateur|Un grain de feuille brille dessus.
+narrateur|Raphaël colle son nez à la vitre.
+narrateur|Le jardin sent la terre mouillée.
+narrateur|La dalle du seau luit, pâle.
 narrateur|Papa ouvre le tiroir de laine.
-narrateur|Ça fait un petit bruit.
-narrateur|Les vitres sont un peu grises.
-narrateur|Une tasse fume près de la fenêtre.
-papa|Raphaël, tu entends la goutte ?
-enfant-m|Oui.
-enfant-m|Je veux l'escargot.
-papa|Il est dans le jardin, tout lent.
+narrateur|Ça fait un petit bruit sourd.
+narrateur|La maison sent la laine et le thé.
+narrateur|Une botte penche près de la porte.
+papa|Raphaël, tu vois le grain dehors ?
+enfant-m|Oui, papa.
+enfant-m|Je veux l'escargot maintenant.
+papa|Sa trace d'argent va sécher.
 papa|On y va, avec le sac.
-narrateur|En ce moment, Raphaël s'accroupit.
+narrateur|En ce moment, Raphaël saisit le sac.
 narrateur|Le sac vert est par terre.
-narrateur|Le tissu est un peu rêche.
+narrateur|Une loupe ronde attend dans la poche.
 enfant-m|Il est vert, papa.
 papa|Oui, c'est le tien.
-papa|Prends de l'eau, même s'il a plu.
-narrateur|Raphaël prend la gourde.
-narrateur|Elle est froide comme la pluie.
-narrateur|Il la met dans le sac.
-papa|Le bonnet aussi, le vent est humide.
-narrateur|Raphaël prend le bonnet.
-narrateur|Il est tout doux.
-narrateur|Il sent la laine du tiroir.
-enfant-m|Il est chaud.
-narrateur|Il le met dans le sac.
-papa|Et le livre, si on s'assoit.
-narrateur|Le livre est près de la tasse.
-narrateur|La couverture est lisse.
-narrateur|Une goutte glisse encore sur la vitre.
-narrateur|Raphaël tire le zip.
-narrateur|Le zip reste un peu.
+papa|Prends la loupe, pour ses cornes.
+narrateur|Raphaël prend la loupe ronde.
+narrateur|Le verre est froid sous le doigt.
+narrateur|Le bord fait un petit clic.
+enfant-m|Vite, il va partir.
+narrateur|Raphaël tape du pied, impatient.
+narrateur|Il pousse la loupe dans le sac.
+narrateur|Il tire le zip d'un coup.
+narrateur|Le zip se coince, dur.
 enfant-m|Ça ne veut pas, papa.
-papa|Doucement, tu aides le zip ?</t>
+narrateur|La loupe bascule et glisse.
+narrateur|Raphaël la rattrape contre sa poitrine.
+narrateur|Son sourire disparaît.
+narrateur|L'envie et l'inquiétude se bousculent.
+narrateur|Le cœur de Raphaël bat plus fort.
+narrateur|Papa s'accroupit à sa hauteur.
+papa|Tu aides le zip ?</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>pluie</t>
+          <t>pluie,tasse,tiroir</t>
         </is>
       </c>
     </row>
@@ -1391,17 +1398,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Raphaël prépare le sac. Où met-il les affaires ?</t>
+          <t>La loupe attend près du zip. Raphaël prépare le sac. Où met-il les affaires ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Raphaël prépare le sac. Où met-il les affaires ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;La loupe attend près du zip. Raphaël prépare le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt;. Où met-il les affaires ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Xavier prépare le &lt;emphasis&gt;sac&lt;/emphasis&gt;. Que fait-il ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;La loupe attend près du zip. Raphaël prépare le &lt;emphasis&gt;sac&lt;/emphasis&gt;. Où met-il les affaires ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1464,7 +1471,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1472,10 +1479,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1490,11 +1497,11 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AH3" s="2" t="inlineStr">
         <is>
@@ -1505,23 +1512,23 @@
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>380</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1530,13 +1537,13 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
@@ -1546,12 +1553,13 @@
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=la_loupe_va_dans_le_sac; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Raphaël prépare le sac.
+          <t>narrateur|La loupe attend près du zip.
+narrateur|Raphaël prépare le sac.
 narrateur|Où met-il les affaires ?</t>
         </is>
       </c>
@@ -1579,17 +1587,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Raphaël pousse encore, tout doux. Le zip avance. Il glisse le livre dans le sac. Il est au chaud. Merci, Raphaël. Raphaël ferme le sac. Ça fait zzz. Le sac vert est fermé. Le sac est prêt ? Oui, papa. Raphaël pose la main sur le sac. Le vert est un peu sombre. Une goutte glisse sur la vitre. Le livre est au chaud, maintenant. Dans le sac. On met le manteau ? Oui.</t>
+          <t>Raphaël refuse de foncer. Il pose la loupe sur le bois. Papa attend, sans parler. Il observe la loupe, puis le zip. Le seau tape un petit tic. Il regarde les dents du zip. Un grain de feuille est coincé. C'est le grain de la feuille. Il le soulève du bout de l'ongle. Le zip se libère, lisse. Il glisse la loupe dans le sac. Le verre rejoint le fond. Elle est au chaud. Merci, Raphaël. Raphaël ferme le sac. Ça fait zzz, bas. Le sac vert est fermé. Le sac est prêt ? Oui, papa. Il pose la main sur le tissu. Le vert est un peu sombre. La vitre montre le seau, dehors. On met le manteau ? Oui.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Raphaël pousse encore, tout doux. Le zip avance. Il glisse le livre dans le sac. Il est au chaud. Merci, Raphaël. Raphaël ferme le sac. Ça fait zzz. Le sac vert est fermé. Le sac est prêt ? Oui, papa. Raphaël pose la main sur le sac. Le vert est un peu sombre. Une goutte glisse sur la vitre. Le livre est au chaud, maintenant. Dans le sac. On met le manteau ? Oui.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Raphaël refuse de foncer. Il pose la loupe sur le bois. Papa attend, sans parler. Il observe la loupe, puis le zip. Le seau tape un petit tic. Il regarde les dents du zip. Un &lt;emphasis level="moderate"&gt;grain de feuille&lt;/emphasis&gt; est coincé. C'est le grain de la feuille. Il le soulève du bout de l'ongle. Le zip se libère, lisse. Il glisse la loupe dans le sac. Le verre rejoint le fond. Elle est au chaud. Merci, Raphaël. Raphaël ferme le sac. Ça fait zzz, bas. Le sac vert est fermé. Le sac est prêt ? Oui, papa. Il pose la main sur le tissu. Le vert est un peu sombre. La vitre montre le seau, dehors. On met le manteau ? Oui.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Xavier a écouté. Il a mis la gourde. Il a mis le bonnet. Il a mis le livre. Le &lt;emphasis&gt;sac&lt;/emphasis&gt; est prêt. C'est ce que l'adulte a dit.&lt;/slow&gt; [pause]</t>
+          <t>Raphaël refuse de foncer. Il pose la loupe sur le bois. Papa attend, sans parler. Il observe la loupe, puis le zip. Le seau tape un petit tic. Il regarde les dents du zip. Un &lt;emphasis&gt;grain de feuille&lt;/emphasis&gt; est coincé. C'est le grain de la feuille. Il le soulève du bout de l'ongle. Le zip se libère, lisse. Il glisse la loupe dans le sac. Le verre rejoint le fond. Elle est au chaud. Merci, Raphaël. Raphaël ferme le sac. Ça fait zzz, bas. Le sac vert est fermé. Le sac est prêt ? Oui, papa. Il pose la main sur le tissu. Le vert est un peu sombre. La vitre montre le seau, dehors. On met le manteau ? Oui. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1636,7 +1644,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>118</v>
+        <v>132</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1644,10 +1652,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.2</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1670,7 +1678,7 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>sac</t>
+          <t>grain de feuille</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
@@ -1680,20 +1688,20 @@
         <v>450</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>380</v>
+        <v>280</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1702,10 +1710,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1714,34 +1722,46 @@
         <v>50</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=confirmation; intention=relancer; emotion=fierté_calme; intensite=1; destinataire=enfant; sous_texte=il_a_refusé_de_foncer; tempo=naturel; sourire=léger; respiration=fluide</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Raphaël pousse encore, tout doux.
-narrateur|Le zip avance.
-narrateur|Il glisse le livre dans le sac.
-enfant-m|Il est au chaud.
+          <t>narrateur|Raphaël refuse de foncer.
+narrateur|Il pose la loupe sur le bois.
+narrateur|Papa attend, sans parler.
+narrateur|Il observe la loupe, puis le zip.
+narrateur|Le seau tape un petit tic.
+narrateur|Il regarde les dents du zip.
+narrateur|Un grain de feuille est coincé.
+enfant-m|C'est le grain de la feuille.
+narrateur|Il le soulève du bout de l'ongle.
+narrateur|Le zip se libère, lisse.
+narrateur|Il glisse la loupe dans le sac.
+narrateur|Le verre rejoint le fond.
+enfant-m|Elle est au chaud.
 papa|Merci, Raphaël.
 narrateur|Raphaël ferme le sac.
-narrateur|Ça fait zzz.
+narrateur|Ça fait zzz, bas.
 narrateur|Le sac vert est fermé.
 papa|Le sac est prêt ?
 enfant-m|Oui, papa.
-narrateur|Raphaël pose la main sur le sac.
+narrateur|Il pose la main sur le tissu.
 narrateur|Le vert est un peu sombre.
-narrateur|Une goutte glisse sur la vitre.
-papa|Le livre est au chaud, maintenant.
-enfant-m|Dans le sac.
+narrateur|La vitre montre le seau, dehors.
 papa|On met le manteau ?
 enfant-m|Oui.</t>
         </is>
       </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>zip,seau</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1766,17 +1786,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Raphaël enfile le manteau. Le manteau sent encore la pluie. Tu as fini ton manteau ? Oui, papa. On ouvre la porte. Papa ouvre la porte. L'air sent la terre mouillée. Le seau a encore sa feuille collée. Une flaque fait un petit cercle. Elle est ronde, papa. Oui, on la regarde. Ils restent un moment. Sous une feuille, un escargot avance. Sa coquille est brillante, un peu brune. Il est là. Tout lent, comme toi tout à l'heure. Une goutte tombe dans la flaque. Le cercle grandit un peu. Encore, papa. On en regarde une autre ? Oui.</t>
+          <t>Raphaël enfile le manteau. Le manteau sent la pluie. Tu as fini ton manteau ? Oui, papa. On ouvre la porte. Papa ouvre la porte. L'air sent la terre mouillée. Le seau garde sa feuille collée. Une flaque fait un petit cercle. Vite, sous toutes les feuilles. Il avance la main trop vite. La feuille glisse, trop loin. Il n'est pas là. Raphaël s'arrête net. Toutes les feuilles se ressemblent. Cette fois, il refuse de foncer. Il cherche le grain de feuille. Le grain brille sur la feuille du seau. C'est lui, papa. Ils s'accroupissent près du seau. La terre est froide sous les genoux. Il soulève le bord, sans brusquer. Sous la feuille, un escargot avance. Sa coquille est brillante, un peu brune. Il est là. Tu l'as trouvé, sans foncer. Une goutte tombe dans la flaque. Le cercle grandit un peu. On le regarde avec la loupe ? Oui.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Raphaël enfile le manteau. Le manteau sent encore la pluie. Tu as fini ton manteau ? Oui, papa. On ouvre la porte. Papa ouvre la porte. L'air sent la terre mouillée. Le seau a encore sa feuille collée. Une flaque fait un petit cercle. Elle est ronde, papa. Oui, on la regarde. Ils restent un moment. Sous une feuille, un escargot avance. Sa coquille est brillante, un peu brune. Il est là. Tout lent, comme toi tout à l'heure. Une goutte tombe dans la flaque. Le cercle grandit un peu. Encore, papa. On en regarde une autre ? Oui.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Raphaël enfile le manteau. Le manteau sent la pluie. Tu as fini ton manteau ? Oui, papa. On ouvre la porte. Papa ouvre la porte. L'air sent la terre mouillée. Le seau garde sa feuille collée. Une flaque fait un petit cercle. Vite, sous toutes les feuilles. Il avance la main trop vite. La feuille glisse, trop loin. Il n'est pas là. Raphaël s'arrête net. Toutes les feuilles se ressemblent. Cette fois, il refuse de foncer. Il cherche le &lt;emphasis level="moderate"&gt;grain de feuille&lt;/emphasis&gt;. Le grain brille sur la feuille du seau. C'est lui, papa. Ils s'accroupissent près du seau. La terre est froide sous les genoux. Il soulève le bord, sans brusquer. Sous la feuille, un escargot avance. Sa coquille est brillante, un peu brune. Il est là. Tu l'as trouvé, sans foncer. Une goutte tombe dans la flaque. Le cercle grandit un peu. On le regarde avec la loupe ? Oui.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Xavier prend le &lt;emphasis&gt;sac&lt;/emphasis&gt;. Papa ouvre la porte. Ils partent.&lt;/slow&gt; [pause]</t>
+          <t>Raphaël enfile le manteau. Le manteau sent la pluie. Tu as fini ton manteau ? Oui, papa. On ouvre la porte. Papa ouvre la porte. L'air sent la terre mouillée. Le seau garde sa feuille collée. Une flaque fait un petit cercle. Vite, sous toutes les feuilles. Il avance la main trop vite. La feuille glisse, trop loin. Il n'est pas là. Raphaël s'arrête net. Toutes les feuilles se ressemblent. Cette fois, il refuse de foncer. Il cherche le &lt;emphasis&gt;grain de feuille&lt;/emphasis&gt;. Le grain brille sur la feuille du seau. C'est lui, papa. Ils s'accroupissent près du seau. La terre est froide sous les genoux. Il soulève le bord, sans brusquer. Sous la feuille, un escargot avance. Sa coquille est brillante, un peu brune. Il est là. Tu l'as trouvé, sans foncer. Une goutte tombe dans la flaque. Le cercle grandit un peu. On le regarde avec la loupe ? Oui. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1823,7 +1843,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>118</v>
+        <v>140</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1831,10 +1851,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1857,30 +1877,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>sac</t>
+          <t>grain de feuille</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>380</v>
+        <v>270</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1889,10 +1909,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1901,32 +1921,50 @@
         <v>50</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=résolution; intention=faire_vivre_la_réussite; emotion=soulagement_joyeux; intensite=2; destinataire=enfant; sous_texte=le_grain_du_début_paie_sous_la_feuille; tempo=naturel; sourire=franc; respiration=relâchée</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
           <t>narrateur|Raphaël enfile le manteau.
-narrateur|Le manteau sent encore la pluie.
+narrateur|Le manteau sent la pluie.
 papa|Tu as fini ton manteau ?
 enfant-m|Oui, papa.
 papa|On ouvre la porte.
 narrateur|Papa ouvre la porte.
 narrateur|L'air sent la terre mouillée.
-narrateur|Le seau a encore sa feuille collée.
+narrateur|Le seau garde sa feuille collée.
 narrateur|Une flaque fait un petit cercle.
-enfant-m|Elle est ronde, papa.
-papa|Oui, on la regarde.
-narrateur|Ils restent un moment.
-narrateur|Sous une feuille, un escargot avance.
+enfant-m|Vite, sous toutes les feuilles.
+narrateur|Il avance la main trop vite.
+narrateur|La feuille glisse, trop loin.
+enfant-m|Il n'est pas là.
+narrateur|Raphaël s'arrête net.
+narrateur|Toutes les feuilles se ressemblent.
+narrateur|Cette fois, il refuse de foncer.
+narrateur|Il cherche le grain de feuille.
+narrateur|Le grain brille sur la feuille du seau.
+enfant-m|C'est lui, papa.
+narrateur|Ils s'accroupissent près du seau.
+narrateur|La terre est froide sous les genoux.
+narrateur|Il soulève le bord, sans brusquer.
+narrateur|Sous la feuille, un escargot avance.
 narrateur|Sa coquille est brillante, un peu brune.
 enfant-m|Il est là.
-papa|Tout lent, comme toi tout à l'heure.
+papa|Tu l'as trouvé, sans foncer.
 narrateur|Une goutte tombe dans la flaque.
 narrateur|Le cercle grandit un peu.
-enfant-m|Encore, papa.
-papa|On en regarde une autre ?
+papa|On le regarde avec la loupe ?
 enfant-m|Oui.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>porte,pluie,flaque</t>
         </is>
       </c>
     </row>
@@ -1953,17 +1991,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>L'escargot pose une corne, puis l'autre. La feuille tremble un tout petit peu. Il avance. Oui, tu l'as trouvé. Le sac vert repose près du seau. Le livre reste au chaud, dedans. Le livre est au chaud, dedans. La flaque ronde brille encore.</t>
+          <t>Raphaël sort la loupe du sac. Le verre encadre deux cornes prudentes. Il avance. Oui, tu l'as trouvé. Le sac vert repose près du seau. La loupe garde une trace d'eau. Le grain de feuille brille toujours. La flaque ronde brille, elle aussi.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>L'escargot pose une corne, puis l'autre. La feuille tremble un tout petit peu. Il avance. Oui, tu l'as trouvé. Le sac vert repose près du seau. Le livre reste au chaud, dedans. Le livre est au chaud, dedans. La flaque ronde brille encore.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Raphaël sort la loupe du sac. Le verre encadre deux cornes prudentes. Il avance. Oui, tu l'as trouvé. Le sac vert repose près du seau. La loupe garde une trace d'eau. Le &lt;emphasis level="moderate"&gt;grain de feuille&lt;/emphasis&gt; brille toujours. La flaque ronde brille, elle aussi.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Raphaël sort la loupe du sac. Le verre encadre deux cornes prudentes. Il avance. Oui, tu l'as trouvé. Le sac vert repose près du seau. La loupe garde une trace d'eau. Le &lt;emphasis&gt;grain de feuille&lt;/emphasis&gt; brille toujours. La flaque ronde brille, elle aussi.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2010,18 +2048,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2030,12 +2068,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2044,17 +2082,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>grain de feuille</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>380</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2063,11 +2105,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2076,31 +2118,35 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=la_loupe_porte_une_trace_d_eau; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|L'escargot pose une corne, puis l'autre.
-narrateur|La feuille tremble un tout petit peu.
+          <t>narrateur|Raphaël sort la loupe du sac.
+narrateur|Le verre encadre deux cornes prudentes.
 enfant-m|Il avance.
 papa|Oui, tu l'as trouvé.
 narrateur|Le sac vert repose près du seau.
-narrateur|Le livre reste au chaud, dedans.
-papa|Le livre est au chaud, dedans.
-narrateur|La flaque ronde brille encore.</t>
+narrateur|La loupe garde une trace d'eau.
+narrateur|Le grain de feuille brille toujours.
+narrateur|La flaque ronde brille, elle aussi.</t>
         </is>
       </c>
     </row>
@@ -2121,7 +2167,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2213,6 +2259,13 @@
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>